<commit_message>
fix: 세금계산서 총액 900,344,264원 (26년 확정 840,514,264 + 25년 59,830,000)
- 바이오힐보 US 30,000,000은 25년 발행분 59,830,000 안에 포함되는 구조로 확정
- 기존 931,288,075는 US를 별도로 한 번 더 더한 값 → 중복 30,000,000, 순 -30,943,811
- 국가 배분: 글로벌 61,796,000(JP 31,796,000 + US 30,000,000) / 국내 838,548,264
  / + JP 미발행 8,904,000 → 진행 기준 909,248,264
- 02_브랜드별: US 행 청구액 비움(25년 계약 행에 포함), 확정 조정 70,431,189 복원
- 03_연월별: 2025~26.01 금액 복원, US는 국가 재배분 행으로만 처리(총계 불변)
- 건당 청구단가 307,481 → 290,531 (2025계약+US 340건/59,830,000 단일 행)
- A4: 국내 2025 계약 272건 대응액 건당 109,669원 확인 항목 추가

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Po6GEYZVM1ncJCBSngkbPu
</commit_message>
<xml_diff>
--- a/reports/올리브영_시딩_성과보고서.xlsx
+++ b/reports/올리브영_시딩_성과보고서.xlsx
@@ -647,7 +647,7 @@
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>집계 26.09.07 · 시딩 2,139건 · 청구 840,514,264원(확정) · 조회수 56,612,765 · 매출 1,420,018,525원</t>
+          <t>집계 26.09.07 · 시딩 2,139건 · 청구 900,344,264원(확정) · 조회수 56,612,765 · 매출 1,420,018,525원</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>840514264</v>
+        <v>900344264</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>307481</v>
+        <v>290531</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
         <v/>
       </c>
       <c r="D13" s="13" t="n">
-        <v>778718264</v>
+        <v>838548264</v>
       </c>
       <c r="E13" s="14">
         <f>D13/$D$16</f>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="I16" s="21" t="inlineStr">
         <is>
-          <t>진행 기준 총계 · 세금계산서 발행 확정 840,514,264 + JP 미발행 8,904,000</t>
+          <t>진행 기준 총계 · 발행 확정 900,344,264 (26년 840,514,264 + 25년 59,830,000) + JP 미발행 8,904,000</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
     <row r="19">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>[금액] 세금계산서 발행 총액 840,514,264원(26.09.07 확정 · 26.02~08 발행분이 전부이며 2025 진행분 정산·바이오힐보 US 포함) 기준</t>
+          <t>[금액] 세금계산서 발행 총액 900,344,264원 = 26.02~08 확정 840,514,264 + 25년 발행 59,830,000(바이오힐보 US 30,000,000 포함)</t>
         </is>
       </c>
     </row>
@@ -1416,9 +1416,7 @@
         <f>SUM(B11:C11)</f>
         <v/>
       </c>
-      <c r="E11" s="27" t="n">
-        <v>30000000</v>
-      </c>
+      <c r="E11" s="27" t="n"/>
       <c r="F11" s="27">
         <f>IFERROR(E11/D11,"")</f>
         <v/>
@@ -1441,7 +1439,7 @@
       </c>
       <c r="L11" s="30" t="inlineStr">
         <is>
-          <t>25.08 US 68건 중 36건 성과 확보</t>
+          <t>25.08 US 68건 중 36건 성과 확보 · 청구 30,000,000은 2025 계약 정산분에 포함</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1816,7 @@
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n">
-        <v>40431189</v>
+        <v>70431189</v>
       </c>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
@@ -1828,7 +1826,7 @@
       <c r="K20" s="25" t="n"/>
       <c r="L20" s="16" t="inlineStr">
         <is>
-          <t>발행 확정 총액 − 프로젝트별 내역 차이 · 브랜드 귀속 확인필요 (A1·A4)</t>
+          <t>26.02~08 발행 확정액 − 프로젝트별 내역 차이 · 브랜드 귀속 확인필요 (A1·A4)</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1839,9 @@
       <c r="B21" s="13" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
+      <c r="E21" s="13" t="n">
+        <v>59830000</v>
+      </c>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
       <c r="H21" s="14" t="n"/>
@@ -1850,7 +1850,7 @@
       <c r="K21" s="25" t="n"/>
       <c r="L21" s="16" t="inlineStr">
         <is>
-          <t>25.04~26.01 진행 272건 · 정산액은 위 확정 총액에 포함 (A3 참조)</t>
+          <t>25.04~26.01 진행 272건 · 바이오힐보 US 30,000,000 포함 · 브랜드 혼재 (A3 참조)</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
         <v/>
       </c>
       <c r="E22" s="18">
-        <f>E19+E20</f>
+        <f>E19+E20+E21</f>
         <v/>
       </c>
       <c r="F22" s="18">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="L22" s="21" t="inlineStr">
         <is>
-          <t>세금계산서 발행 확정 840,514,264원과 일치</t>
+          <t>세금계산서 발행 확정 900,344,264원과 일치</t>
         </is>
       </c>
     </row>
@@ -1923,14 +1923,14 @@
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>· 바이오힐보 US 68건은 청구 30,000,000원 전액을 계상하고 조회수는 성과 확보 36건분(4,739,117뷰)만 넣었다. 건당 조회수는 국내의 4.7배.</t>
+          <t>· 바이오힐보 US 68건의 청구 30,000,000원은 2025 시딩 계약 행에 포함돼 있다. 조회수는 성과 확보 36건분(4,739,117뷰)이며 건당 조회수는 국내의 4.7배.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="22" t="inlineStr">
         <is>
-          <t>· 2025 시딩 계약(272건)의 정산액 59,830,000원은 26.02~08 발행 확정 총액 안에 포함되어 있어 별도 금액으로 더하지 않는다. 수량은 IMD 반영분(53건)만 위 브랜드에 들어가 있다.</t>
+          <t>· 2025 시딩 계약 정산액 59,830,000원에는 바이오힐보 US 30,000,000원이 포함되어 있다. 따라서 US 행의 청구 금액은 비웠고, 수량은 IMD 반영분(53건)만 위 브랜드에 들어가 있다.</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,9 @@
         <f>SUM(B6:D6)</f>
         <v/>
       </c>
-      <c r="F6" s="13" t="n"/>
+      <c r="F6" s="13" t="n">
+        <v>7300000</v>
+      </c>
       <c r="G6" s="13" t="n"/>
       <c r="H6" s="13">
         <f>SUM(F6:G6)</f>
@@ -2392,7 +2394,7 @@
       </c>
       <c r="M6" s="16" t="inlineStr">
         <is>
-          <t>2025 계약 진행 (식물나라 51건) · 정산은 26년 발행</t>
+          <t>2025 계약 진행 (식물나라 51건)</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2411,9 @@
         <f>SUM(B7:D7)</f>
         <v/>
       </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="F7" s="13" t="n">
+        <v>12215000</v>
+      </c>
       <c r="G7" s="13" t="n"/>
       <c r="H7" s="13">
         <f>SUM(F7:G7)</f>
@@ -2424,7 +2428,7 @@
       </c>
       <c r="M7" s="16" t="inlineStr">
         <is>
-          <t>2025 계약 진행 (44건) · 정산은 26년 발행</t>
+          <t>2025 계약 진행 (44건)</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2447,9 @@
         <f>SUM(B8:D8)</f>
         <v/>
       </c>
-      <c r="F8" s="13" t="n"/>
+      <c r="F8" s="13" t="n">
+        <v>19315000</v>
+      </c>
       <c r="G8" s="13" t="n"/>
       <c r="H8" s="13">
         <f>SUM(F8:G8)</f>
@@ -2460,7 +2466,7 @@
       </c>
       <c r="M8" s="16" t="inlineStr">
         <is>
-          <t>2025 계약 77건 + 바이오힐보 US 68건 · 정산은 26년 발행</t>
+          <t>2025 계약 77건 + 바이오힐보 US 68건</t>
         </is>
       </c>
     </row>
@@ -2515,7 +2521,9 @@
         <f>SUM(B10:D10)</f>
         <v/>
       </c>
-      <c r="F10" s="13" t="n"/>
+      <c r="F10" s="13" t="n">
+        <v>11760000</v>
+      </c>
       <c r="G10" s="13" t="n"/>
       <c r="H10" s="13">
         <f>SUM(F10:G10)</f>
@@ -2530,11 +2538,7 @@
         <f>IFERROR(K10/J10,"")</f>
         <v/>
       </c>
-      <c r="M10" s="16" t="inlineStr">
-        <is>
-          <t>정산은 26년 발행</t>
-        </is>
-      </c>
+      <c r="M10" s="16" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
@@ -2551,7 +2555,9 @@
         <f>SUM(B11:D11)</f>
         <v/>
       </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="F11" s="13" t="n">
+        <v>8190000</v>
+      </c>
       <c r="G11" s="13" t="n"/>
       <c r="H11" s="13">
         <f>SUM(F11:G11)</f>
@@ -2566,11 +2572,7 @@
         <f>IFERROR(K11/J11,"")</f>
         <v/>
       </c>
-      <c r="M11" s="16" t="inlineStr">
-        <is>
-          <t>정산은 26년 발행</t>
-        </is>
-      </c>
+      <c r="M11" s="16" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
@@ -2619,7 +2621,9 @@
         <f>SUM(B13:D13)</f>
         <v/>
       </c>
-      <c r="F13" s="13" t="n"/>
+      <c r="F13" s="13" t="n">
+        <v>1050000</v>
+      </c>
       <c r="G13" s="13" t="n"/>
       <c r="H13" s="13">
         <f>SUM(F13:G13)</f>
@@ -2638,11 +2642,7 @@
         <f>IFERROR(K13/J13,"")</f>
         <v/>
       </c>
-      <c r="M13" s="16" t="inlineStr">
-        <is>
-          <t>정산은 26.02 이후 발행</t>
-        </is>
-      </c>
+      <c r="M13" s="16" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
@@ -2949,7 +2949,7 @@
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>(발행월 미확정)</t>
+          <t>(국가 재배분)</t>
         </is>
       </c>
       <c r="B21" s="13" t="n"/>
@@ -2978,7 +2978,7 @@
       </c>
       <c r="M21" s="16" t="inlineStr">
         <is>
-          <t>바이오힐보 US 30,000,000 국가 재배분 (금액 총계 불변)</t>
+          <t>바이오힐보 US 30,000,000 · 2025 계약 금액에 포함되어 있어 KR→글로벌 이동 (총계 불변)</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="M23" s="21" t="inlineStr">
         <is>
-          <t>금액 849,418,264 = 발행 확정 840,514,264 + JP 미발행 8,904,000</t>
+          <t>금액 909,248,264 = 발행 확정 900,344,264 + JP 미발행 8,904,000</t>
         </is>
       </c>
     </row>
@@ -3084,14 +3084,14 @@
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>· 26.02~08 월별 금액은 26.09.07 확정 총액표를 그대로 반영했고, 이 7개월분이 세금계산서 발행액 전부다. 2025 진행분 정산·바이오힐보 US도 이 안에 포함된다.</t>
+          <t>· 26.02~08 월별 금액은 26.09.07 확정 총액표 그대로다. 여기에 2025 발행분 59,830,000(25.04~26.01 진행분 정산)을 더한 900,344,264원이 총 발행액이다.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="22" t="inlineStr">
         <is>
-          <t>· 바이오힐보 US 30,000,000원은 발행월이 특정되지 않아 국가 배분만 별도 행으로 조정했다(KR −30,000,000 / 글로벌 +30,000,000, 총계 불변).</t>
+          <t>· 바이오힐보 US 30,000,000원은 2025 계약 금액 안에 있어 국가 배분만 별도 행으로 조정했다(KR −30,000,000 / 글로벌 +30,000,000, 총계 불변).</t>
         </is>
       </c>
     </row>
@@ -4188,16 +4188,16 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>840514264</v>
+        <v>900344264</v>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>26.02~08 발행분이 전부. 2025 진행분 정산 59,830,000 · 바이오힐보 US 30,000,000도 이 안에 포함</t>
+          <t>26.02~08 확정 840,514,264 + 25년 발행 59,830,000 (바이오힐보 US 30,000,000 포함)</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>— 아래 참조</t>
+          <t>420,918원 ≠ 건당단가</t>
         </is>
       </c>
     </row>
@@ -4208,11 +4208,11 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>-90773811</v>
+        <v>-30943811</v>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>기존 931,288,075은 25년 발행분 89,830,000을 별도로 더한 값 → 확정 총액에 이미 포함되어 있어 중복</t>
+          <t>기존 931,288,075은 US 30,000,000을 25년 발행분과 별도로 더한 값 → 중복. 여기에 26년 확정 −943,811 반영</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr"/>
@@ -4240,7 +4240,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>849418264</v>
+        <v>909248264</v>
       </c>
       <c r="C16" s="16" t="inlineStr"/>
       <c r="D16" s="16" t="inlineStr"/>
@@ -4284,7 +4284,7 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>③ 건당 청구단가 307,481원 — 산정 근거</t>
+          <t>③ 건당 청구단가 290,531원 — 산정 근거</t>
         </is>
       </c>
     </row>
@@ -4364,14 +4364,14 @@
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>바이오힐보 US</t>
+          <t>2025 시딩 계약 + 바이오힐보 US</t>
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>68</v>
+        <v>340</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>30000000</v>
+        <v>59830000</v>
       </c>
       <c r="D25" s="13">
         <f>IFERROR(C25/B25,"")</f>
@@ -4379,66 +4379,56 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>2025 시딩 계약</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="n">
-        <v>272</v>
-      </c>
-      <c r="C26" s="13" t="n">
-        <v>59830000</v>
-      </c>
-      <c r="D26" s="13">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>가중평균</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>SUM(B22:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="18">
+        <f>SUM(C22:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="18">
         <f>IFERROR(C26/B26,"")</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>가중평균</t>
-        </is>
-      </c>
-      <c r="B27" s="18">
-        <f>SUM(B22:B26)</f>
-        <v/>
-      </c>
-      <c r="C27" s="18">
-        <f>SUM(C22:C26)</f>
-        <v/>
-      </c>
-      <c r="D27" s="18">
-        <f>IFERROR(C27/B27,"")</f>
-        <v/>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>· 분자·분모가 같은 자료에서 함께 확정되는 항목만 사용 (전체 청구액의 57%, 진행 1,770건).</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
         <is>
-          <t>· 분자·분모가 같은 자료에서 함께 확정되는 항목만 사용 (전체 청구액의 65%, 진행 1,770건).</t>
+          <t>· 검증 1 — 아포맨 대조표 296,750,000 + 지급대행 5,000,000 = 세금계산서 발행 2~7월 301,750,000 (일치).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="22" t="inlineStr">
         <is>
-          <t>· 검증 1 — 아포맨 대조표 296,750,000 + 지급대행 5,000,000 = 세금계산서 발행 2~7월 301,750,000 (일치).</t>
+          <t>· 검증 2 — 아포맨 원고료 272,248원 × 마크업 1.25 = 340,310원 = 실제 청구 단가 (일치).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="22" t="inlineStr">
         <is>
-          <t>· 검증 2 — 아포맨 원고료 272,248원 × 마크업 1.25 = 340,310원 = 실제 청구 단가 (일치).</t>
+          <t>· 총액 900,344,264 ÷ 2,139 = 420,918원은 건당 단가가 아니다. 분자에 비시딩 항목이 있고, 청구 대응 진행 건수(약 2,787건)가 분모보다 크다.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="22" t="inlineStr">
         <is>
-          <t>· 총액 840,514,264 ÷ 2,139 = 392,948원은 건당 단가가 아니다. 분자에 비시딩 항목이 있고, 청구 대응 진행 건수(약 2,787건)가 분모보다 크다.</t>
+          <t>· 2025 계약 59,830,000원에 바이오힐보 US 30,000,000원이 포함되므로 국내 272건에 대응하는 금액은 29,830,000원(건당 109,669원)이 된다. 나노 단가(25만원)보다 낮아 272건 중 일부는 무상·재사용 건일 가능성이 있다 → A4 확인 항목.</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5168,24 +5158,24 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>세금계산서 총액 (발행 확정)</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>26.02~08</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="18" t="n"/>
-      <c r="I25" s="18" t="n"/>
-      <c r="J25" s="18">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>2026.02~08 발행 확정</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>구분 없음</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13">
         <f>J6</f>
         <v/>
       </c>
@@ -5193,12 +5183,12 @@
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  글로벌 · 일본(JP) 발행분</t>
+          <t>25.04~26.01  2025 발행분 (272건 + US 68건)</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>일본(JP)</t>
+          <t>국내+US</t>
         </is>
       </c>
       <c r="C26" s="13" t="n"/>
@@ -5209,63 +5199,59 @@
       <c r="H26" s="13" t="n"/>
       <c r="I26" s="13" t="n"/>
       <c r="J26" s="13" t="n">
+        <v>59830000</v>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>세금계산서 총액 (발행 확정)</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="inlineStr"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18">
+        <f>J25+J26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  글로벌 · 일본(JP) 발행분</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>일본(JP)</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n">
         <v>31796000</v>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  글로벌 · 바이오힐보 US</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>미국(US)</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n">
-        <v>30000000</v>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  국내 (KR) = 총액 − 글로벌</t>
-        </is>
-      </c>
-      <c r="B28" s="37" t="inlineStr">
-        <is>
-          <t>국내</t>
-        </is>
-      </c>
-      <c r="C28" s="32" t="n"/>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="32" t="n"/>
-      <c r="G28" s="32" t="n"/>
-      <c r="H28" s="32" t="n"/>
-      <c r="I28" s="32" t="n"/>
-      <c r="J28" s="32">
-        <f>J25-J26-J27</f>
-        <v/>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  + JP 미발행 (26.09)</t>
+          <t xml:space="preserve">  글로벌 · 바이오힐보 US (25년 발행분에 포함)</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>일본(JP)</t>
+          <t>미국(US)</t>
         </is>
       </c>
       <c r="C29" s="13" t="n"/>
@@ -5276,58 +5262,103 @@
       <c r="H29" s="13" t="n"/>
       <c r="I29" s="13" t="n"/>
       <c r="J29" s="13" t="n">
+        <v>30000000</v>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  국내 (KR) = 총액 − 글로벌</t>
+        </is>
+      </c>
+      <c r="B30" s="37" t="inlineStr">
+        <is>
+          <t>국내</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="n"/>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="32" t="n"/>
+      <c r="F30" s="32" t="n"/>
+      <c r="G30" s="32" t="n"/>
+      <c r="H30" s="32" t="n"/>
+      <c r="I30" s="32" t="n"/>
+      <c r="J30" s="32">
+        <f>J27-J28-J29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + JP 미발행 (26.09)</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>일본(JP)</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="13" t="n"/>
+      <c r="F31" s="13" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="n"/>
+      <c r="J31" s="13" t="n">
         <v>8904000</v>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="17" t="inlineStr">
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>진행 기준 총계</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="18" t="n"/>
-      <c r="I30" s="18" t="n"/>
-      <c r="J30" s="18">
-        <f>J25+J29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>· 26.02~08 확정 총액 840,514,264원이 세금계산서 발행액 전부다. 2025 진행분 정산(59,830,000)과 바이오힐보 US(30,000,000)도 이 안에 포함되어 있어 별도로 더하지 않는다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="22" t="inlineStr">
-        <is>
-          <t>· 기존 집계 931,288,075원은 위 두 항목을 확정 총액에 다시 더한 값이었다 (중복 89,830,000). 정정 후 −90,773,811원.</t>
-        </is>
+      <c r="B32" s="20" t="inlineStr"/>
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="18" t="n"/>
+      <c r="F32" s="18" t="n"/>
+      <c r="G32" s="18" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="18" t="n"/>
+      <c r="J32" s="18">
+        <f>J27+J31</f>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="22" t="inlineStr">
         <is>
-          <t>· 확정 반영으로 빠진 것 — 26.02 아이디얼포맨 계상분 71,375,000원 (확정 2월 92,750,000원은 루테카 단독과 일치).</t>
+          <t>· 총 발행액 900,344,264원 = 26.02~08 확정 840,514,264 + 25년 발행 59,830,000. 25년 발행분 안에 바이오힐보 US 30,000,000원이 포함되어 있다.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="22" t="inlineStr">
         <is>
-          <t>· 프로젝트별 내역(②) 대비 차액 70,431,189원 — 2025 계약 정산분·US 청구분(합 89,830,000)의 일부가 여기에, 나머지는 이미 ②의 프로젝트 라인에 계상된 것으로 보인다. 정확한 귀속은 확인 필요.</t>
+          <t>· 기존 집계 931,288,075원은 US 30,000,000원을 25년 발행분과 별도로 한 번 더 더한 값이었다 → 중복 30,000,000. 여기에 26년 확정 −943,811을 반영해 순 −30,943,811원.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>· 확정 반영으로 빠진 것 — 26.02 아이디얼포맨 계상분 71,375,000원 (확정 2월 92,750,000원은 루테카 단독과 일치).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>· 확정 반영으로 더해진 것 — 26.03 +42,075,000 / 26.04 +5,058,689 / 26.05 +22,553,250 / 26.08 +31,740,500, 26.07 −30,996,250 (7→8월 발행 이동 추정) → 순 +70,431,189. 프로젝트별 귀속은 확인 필요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>· 총액표에 국가 구분이 없어 글로벌 시딩 라인 자료로 귀속했다. 루테카·바이오힐보는 분리 근거가 없어 혼재로 둔다.</t>
         </is>
@@ -7036,7 +7067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7098,7 +7129,7 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>발행 확정 총액이 프로젝트별 내역보다 70,431,189원 많다(US 30,000,000 제외 시 40,431,189). 2025 계약 정산분·US 청구분 포함 여부와 프로젝트별 귀속 확인 필요</t>
+          <t>26.02~08 발행 확정액이 프로젝트별 내역보다 70,431,189원 많다(03 +42,075,000 / 04 +5,058,689 / 05 +22,553,250 / 07 −30,996,250 / 08 +31,740,500). 프로젝트별 귀속 필요</t>
         </is>
       </c>
       <c r="D5" s="13" t="n">
@@ -7112,19 +7143,21 @@
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>청구 대응 진행 건수</t>
+          <t>2025 계약 국내 건당액</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>세금계산서에 수량 미기재 → 840,514,264원에 대응하는 진행 건수 확정 불가(추정 약 2,787건). 확정 시 건당 단가 확정 가능</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="n"/>
+          <t>59,830,000원에 US 30,000,000원이 포함되므로 국내 272건 대응액은 29,830,000원(건당 109,669원). 나노 단가 25만원보다 낮아 272건 중 무상·재사용 건 포함 여부 확인 필요</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>29830000</v>
+      </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
           <t>높음</t>
@@ -7133,16 +7166,16 @@
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>IMD 국가 분류 오류</t>
+          <t>청구 대응 진행 건수</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>IMD는 일본 24건(WM 9·CG 8·BOH 7)만 분류하나 실제 99건. 54건(WM 30·CG 24)이 국내로 오분류</t>
+          <t>세금계산서에 수량 미기재 → 900,344,264원에 대응하는 진행 건수 확정 불가(추정 약 2,787건). 확정 시 건당 단가 확정 가능</t>
         </is>
       </c>
       <c r="D7" s="13" t="n"/>
@@ -7154,16 +7187,16 @@
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>바이오힐보 국내 비용 귀속</t>
+          <t>IMD 국가 분류 오류</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>국내 195건·원고료 37,900,000인데 26년 발행액은 6,687,500뿐. 2025 계약 + 브랜드사 직계약으로 분산 추정</t>
+          <t>IMD는 일본 24건(WM 9·CG 8·BOH 7)만 분류하나 실제 99건. 54건(WM 30·CG 24)이 국내로 오분류</t>
         </is>
       </c>
       <c r="D8" s="13" t="n"/>
@@ -7175,21 +7208,19 @@
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>식물나라 소계 오류</t>
+          <t>바이오힐보 국내 비용 귀속</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>원본 대조표 소계(384건 / 68,177,200 / 95,145,250)가 구버전(370건) 값. 재계산 시 87,676,850 / 106,723,250</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>11578000</v>
-      </c>
+          <t>국내 195건·원고료 37,900,000인데 26년 발행액은 6,687,500뿐. 2025 계약 + 브랜드사 직계약으로 분산 추정</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n"/>
       <c r="E9" s="16" t="inlineStr">
         <is>
           <t>높음</t>
@@ -7198,20 +7229,20 @@
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>아포맨 누계 행 상충</t>
+          <t>식물나라 소계 오류</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>요약 행에 194,450,000 / 308,887,500 / 243,062,500 세 값 동시 기재. 월별 상세(237,400,000 / 296,750,000)가 정답</t>
+          <t>원본 대조표 소계(384건 / 68,177,200 / 95,145,250)가 구버전(370건) 값. 재계산 시 87,676,850 / 106,723,250</t>
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>12137500</v>
+        <v>11578000</v>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
@@ -7221,43 +7252,43 @@
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>JP 마크업률 미확정</t>
+          <t>아포맨 누계 행 상충</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>JP 고정비 29,465,000만 글로벌로 귀속. 세금계산서 42,292,500과의 차액 약 12.8백만(마크업·VAT)은 KR에 잔류</t>
+          <t>요약 행에 194,450,000 / 308,887,500 / 243,062,500 세 값 동시 기재. 월별 상세(237,400,000 / 296,750,000)가 정답</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>12827500</v>
+        <v>12137500</v>
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>중</t>
+          <t>높음</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>색조 3사 국내분 미발행</t>
+          <t>JP 마크업률 미확정</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>WM 국내 70건·CG 45건·FM 27건의 국내 시딩 비용이 26년 발행액에 없음. 하반기 계약으로 26.09 이후 발행 예정인지 확인</t>
+          <t>JP 고정비 29,465,000만 글로벌로 귀속. 세금계산서 42,292,500과의 차액 약 12.8백만(마크업·VAT)은 KR에 잔류</t>
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>34300000</v>
+        <v>12827500</v>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
@@ -7267,19 +7298,21 @@
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>비시딩 항목 전체 목록</t>
+          <t>색조 3사 국내분 미발행</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>지급대행·모션그래픽·솔루션 32,400,000원은 확인분만. 전체 목록 확보 시 건당 단가 정밀화</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="n"/>
+          <t>WM 국내 70건·CG 45건·FM 27건의 국내 시딩 비용이 26년 발행액에 없음. 하반기 계약으로 26.09 이후 발행 예정인지 확인</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>34300000</v>
+      </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
           <t>중</t>
@@ -7288,16 +7321,16 @@
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>2025년 상반기 데이터</t>
+          <t>비시딩 항목 전체 목록</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>IMD가 25.09.29부터라 25년 1~9월 업로드 데이터 없음. 2025 계약 272건 중 219건이 성과 집계 밖</t>
+          <t>지급대행·모션그래픽·솔루션 32,400,000원은 확인분만. 전체 목록 확보 시 건당 단가 정밀화</t>
         </is>
       </c>
       <c r="D14" s="13" t="n"/>
@@ -7309,63 +7342,61 @@
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>루테카 US 수량</t>
+          <t>2025년 상반기 데이터</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>US TikTok 약 20건이 IMD·세금계산서 어느 쪽에서도 특정되지 않아 집계 제외</t>
+          <t>IMD가 25.09.29부터라 25년 1~9월 업로드 데이터 없음. 2025 계약 272건 중 219건이 성과 집계 밖</t>
         </is>
       </c>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>중</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="12" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>바이오힐보 US 미집계 32건</t>
+          <t>루테카 US 수량</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>US 68건 중 36건만 성과 확보(4,739,117뷰). 나머지 32건 조회수·참여 데이터 미확보 → 실제 성과는 현재 수치 이상</t>
+          <t>US TikTok 약 20건이 IMD·세금계산서 어느 쪽에서도 특정되지 않아 집계 제외</t>
         </is>
       </c>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="16" t="inlineStr">
         <is>
-          <t>중</t>
+          <t>낮음</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>바이오힐보 US 원고료</t>
+          <t>바이오힐보 US 미집계 32건</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>US 36건 원고료 미기재. 청구 30,000,000원만 확인되어 CPV는 청구 기준으로 산출(국내·JP와 기준 상이)</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="n">
-        <v>30000000</v>
-      </c>
+          <t>US 68건 중 36건만 성과 확보(4,739,117뷰). 나머지 32건 조회수·참여 데이터 미확보 → 실제 성과는 현재 수치 이상</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n"/>
       <c r="E17" s="16" t="inlineStr">
         <is>
           <t>중</t>
@@ -7374,47 +7405,47 @@
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>바이오힐보 US 원고료</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>US 36건 원고료 미기재. 청구 30,000,000원만 확인되어 CPV는 청구 기준으로 산출(국내·JP와 기준 상이)</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>케어플러스 청구 차이</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>협의 비용 합 7,825,000(+VAT 8,607,500) vs 세금계산서 8,998,750 → 391,250 차이</t>
         </is>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D19" s="13" t="n">
         <v>391250</v>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>낮음</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="26" t="inlineStr">
-        <is>
-          <t>해결</t>
-        </is>
-      </c>
-      <c r="B19" s="38" t="inlineStr">
-        <is>
-          <t>루테카 발행액 71,375,000</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t>26.02 확정액이 92,750,000(루테카 단독)으로 확정되어 아이디얼포맨 2월 계상분 71,375,000은 제외 확정</t>
-        </is>
-      </c>
-      <c r="D19" s="27" t="n"/>
-      <c r="E19" s="30" t="inlineStr">
-        <is>
-          <t>완료</t>
         </is>
       </c>
     </row>
@@ -7426,12 +7457,12 @@
       </c>
       <c r="B20" s="38" t="inlineStr">
         <is>
-          <t>케어플러스 원고료</t>
+          <t>루테카 발행액 71,375,000</t>
         </is>
       </c>
       <c r="C20" s="30" t="inlineStr">
         <is>
-          <t>시딩현황에서 확인 — 마이크로 5건×200,000 + 나노 27건×100,000 = 3,700,000원. CPV 19.63원 / CPE 2,012원</t>
+          <t>26.02 확정액이 92,750,000(루테카 단독)으로 확정되어 아이디얼포맨 2월 계상분 71,375,000은 제외 확정</t>
         </is>
       </c>
       <c r="D20" s="27" t="n"/>
@@ -7449,12 +7480,12 @@
       </c>
       <c r="B21" s="38" t="inlineStr">
         <is>
-          <t>바이오힐보 US 성과</t>
+          <t>케어플러스 원고료</t>
         </is>
       </c>
       <c r="C21" s="30" t="inlineStr">
         <is>
-          <t>IMD 26.09.07로 36건 확보 — 4,739,117뷰 / 좋아요 23,068 / 댓글 1,066 / 최대 2,954,129뷰(전체 1위)</t>
+          <t>시딩현황에서 확인 — 마이크로 5건×200,000 + 나노 27건×100,000 = 3,700,000원. CPV 19.63원 / CPE 2,012원</t>
         </is>
       </c>
       <c r="D21" s="27" t="n"/>
@@ -7464,8 +7495,31 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="22" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>바이오힐보 US 성과</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>IMD 26.09.07로 36건 확보 — 4,739,117뷰 / 좋아요 23,068 / 댓글 1,066 / 최대 2,954,129뷰(전체 1위)</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>· 금액 영향은 미설명·수정 필요 금액의 절대값이며 서로 중복될 수 있어 합산하지 않는다.</t>
         </is>

</xml_diff>